<commit_message>
Update leads database: 43 verified pan-India leads
</commit_message>
<xml_diff>
--- a/AGMIDI_India_Leads.xlsx
+++ b/AGMIDI_India_Leads.xlsx
@@ -38,7 +38,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +69,12 @@
         <bgColor rgb="004C1D95"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -96,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,6 +121,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -481,22 +499,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="39" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="43" customWidth="1" min="10" max="10"/>
+    <col width="33" customWidth="1" min="9" max="9"/>
+    <col width="53" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="27" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="29" customWidth="1" min="16" max="16"/>
@@ -2627,6 +2645,1497 @@
       <c r="Q25" s="3" t="inlineStr">
         <is>
           <t>Technical analysis, options strategies and live market mentoring sessions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>AGM-1026</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>List of Best Top 10 IIT-JEE NEET Coaching Institutes in Kota</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Kota</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Rajasthan</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>9694580746</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/919694580746</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>info@motion.ac.in</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>https://motion.ac.in/examinfo/list-of-the-best-top-10-iit-jee-neet-coaching-institutes-in-kota/</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Tier A (High Value)</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>Top 10 IIT andNEETCoachingInstitutesinKota:Kota, as a city, has built a strong reputation in India as one of the top education hubs. Thousands of students visit (idioms dictionary)Kotaevery year to prepare for exams likeJEE(Main + Advanced) andNEET. With time, lots ofcoachinginstitutions have grown …</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>AGM-1027</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Top 10 IIT JEE Coaching Institutes in Kota: Fees &amp; Contact Details</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Kota</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Rajasthan</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr"/>
+      <c r="H27" s="8" t="inlineStr"/>
+      <c r="I27" s="8" t="inlineStr"/>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>https://blog.shikshacoach.com/iit-jee-coaching-in-kota/</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>Tier C (Nurture)</t>
+        </is>
+      </c>
+      <c r="M27" s="8" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N27" s="7" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O27" s="7" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P27" s="8" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q27" s="8" t="inlineStr">
+        <is>
+          <t>We mentioned below all the TopCoachingcentres withContactdetails. Top 10BestIITJEEOnlineCoachingin India Rana Sir Classes |BestIITJEECoachinginKotaRana Sir Classes has emerged as a leadingcoachinginstituteinKota, offering comprehensivecoachingprograms for IITJEEaspirants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>AGM-1028</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Kota</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Rajasthan</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>7810060367</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/917810060367</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>admissions@kotaneetacademy.in</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>https://kotaneetacademy.in/</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Tier A (High Value)</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>With years of experience and a foundation built inKota'scoachingexcellence, we specialize in preparing students forNEETandJEE. Our expert mentors, focused approach, and result-driven methods help thousands of aspirants reach their academic goals each year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>AGM-1029</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Aakash Institute</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Kota</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Rajasthan</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>9442441175</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/919442441175</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>kota@aesl.in</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>https://centers.aakash.ac.in/aakash-institute-best-neet-iit-jee-coaching-in-kota-ipia-coaching-center-ipia-kota-276037/Home</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Tier A (High Value)</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>AakashInstitute,Kota, Indraprastha Industrial Area,Kota- Fee Structure, Reviews andContactDetails.BestCoachingin Indraprastha Industrial Area,KotaforNEET&amp; IIT-JEE. Connect with us at 928942xxxx. Get Accurate Address,PhoneNo and Timings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>AGM-1030</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>NEET Coaching Centers in Kota Rajasthan</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Kota</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>Rajasthan</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr"/>
+      <c r="H30" s="10" t="inlineStr"/>
+      <c r="I30" s="10" t="inlineStr"/>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t>https://www.justdial.com/Kota-Rajasthan/Neet-Tutorials/nct-11037560</t>
+        </is>
+      </c>
+      <c r="K30" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="L30" s="9" t="inlineStr">
+        <is>
+          <t>Tier C (Nurture)</t>
+        </is>
+      </c>
+      <c r="M30" s="10" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N30" s="9" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O30" s="9" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P30" s="10" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q30" s="10" t="inlineStr">
+        <is>
+          <t>271NeetTutorials inKotaRajasthan. FindNEETCoachingClasses,NEETEntranceCoaching,NEETCoachingInstitutes, Pre-MedicalNEETUGCoachinginKotaRajasthan. GetPhoneNumbers, Address, Reviews, Photos, Maps for topNeetTutorials near me inKotaRajasthan on Justdial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>AGM-1031</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Best JEE &amp; NEET Coaching in Delhi (150+ Institutes)</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Delhi NCR</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr"/>
+      <c r="H31" s="8" t="inlineStr"/>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>contact@jeeandneet.com</t>
+        </is>
+      </c>
+      <c r="J31" s="8" t="inlineStr">
+        <is>
+          <t>https://jeeandneet.com/coaching/city/Delhi</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="L31" s="7" t="inlineStr">
+        <is>
+          <t>Tier B (Medium Value)</t>
+        </is>
+      </c>
+      <c r="M31" s="8" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O31" s="7" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P31" s="8" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q31" s="8" t="inlineStr">
+        <is>
+          <t>Browse 150+JEE&amp;NEETcoachinginstitutesinDelhi— names, locations andcontactdetails in one place. A free, unbiased directory from JEEandNEET.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>AGM-1032</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Best Coaching Centers in Delhi (2026)</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Delhi NCR</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr"/>
+      <c r="H32" s="10" t="inlineStr"/>
+      <c r="I32" s="10" t="inlineStr"/>
+      <c r="J32" s="10" t="inlineStr">
+        <is>
+          <t>https://www.tuition.in/coaching-centers/delhi/</t>
+        </is>
+      </c>
+      <c r="K32" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="L32" s="9" t="inlineStr">
+        <is>
+          <t>Tier C (Nurture)</t>
+        </is>
+      </c>
+      <c r="M32" s="10" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N32" s="9" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O32" s="9" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P32" s="10" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q32" s="10" t="inlineStr">
+        <is>
+          <t>Home /CoachingCenters /DelhiBestCoachingCenters inDelhiFind and compare the topcoachingcenters inDelhi. CBSE, ICSE,JEE,NEETpreparation with verified ratings, real reviews, and transparent fee information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>AGM-1033</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>NEET Coaching Centers in Delhi</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Delhi NCR</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr"/>
+      <c r="H33" s="8" t="inlineStr"/>
+      <c r="I33" s="8" t="inlineStr"/>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>https://www.justdial.com/Delhi/Neet-Tutorials/nct-11037560</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>Tier C (Nurture)</t>
+        </is>
+      </c>
+      <c r="M33" s="8" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N33" s="7" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O33" s="7" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P33" s="8" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q33" s="8" t="inlineStr">
+        <is>
+          <t>2653NeetTutorials inDelhi. FindNEETCoachingClasses,NEETEntranceCoaching,NEETCoachingInstitutes, Pre-MedicalNEET(UG)CoachinginDelhi. GetPhoneNumbers, Address, Reviews, Photos, Maps for topNeetTutorials near me inDelhion Justdial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>AGM-1034</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Top NEET Coaching Institutes in New Delhi, Contact ...</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Delhi NCR</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>7490196078</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/917490196078</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>https://collegedunia.com/coaching/neet-institutes-in-new-delhi</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Tier A (High Value)</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>TopNEETCoachingInstitutesin NewDelhi. View course-specificinstitutesalong with cost, scholarships and reviews.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>AGM-1035</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Full List of Coaching Institutes in Delhi for Exam Prep</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Delhi NCR</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>7548020221</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/917548020221</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>topcoachingindelhi@gmail.com</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>https://topcoachingindelhi.com/coachings/</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Tier A (High Value)</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P35" s="3" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>CoachingInstitutesinDelhiNCRDiscoverDelhi'spremiercoachinginstitutesfor competitive exams such as UPSC, SSC,NEET,JEE, CUET, UGC‑NET, CLAT, NATA, and Judiciary. Expertly curated, this page provides a well-organized directory of topcoachingcenters, grouped by exam type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>AGM-1036</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>Best JEE &amp; NEET Coaching in Patna (241+ Institutes)</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>Patna</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>Bihar</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr"/>
+      <c r="H36" s="10" t="inlineStr"/>
+      <c r="I36" s="10" t="inlineStr">
+        <is>
+          <t>contact@jeeandneet.com</t>
+        </is>
+      </c>
+      <c r="J36" s="10" t="inlineStr">
+        <is>
+          <t>https://jeeandneet.com/coaching/city/Patna</t>
+        </is>
+      </c>
+      <c r="K36" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="L36" s="9" t="inlineStr">
+        <is>
+          <t>Tier B (Medium Value)</t>
+        </is>
+      </c>
+      <c r="M36" s="10" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N36" s="9" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O36" s="9" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P36" s="10" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q36" s="10" t="inlineStr">
+        <is>
+          <t>Browse 241+JEE&amp;NEETcoachinginstitutesinPatna— names, locations andcontactdetails in one place. A free, unbiased directory from JEEandNEET.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>AGM-1037</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Top 20 IIT JEE Coaching in Patna</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Patna</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Bihar</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>8563888889</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/918563888889</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr"/>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.justdial.com/Patna/Tutorials-For-IIT-JEE/nct-10502810</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Tier A (High Value)</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P37" s="3" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>870 IITJEECoachinginPatna. Find IITJEECoachingClasses, IIT Tutorials, IITJEECoachingCentres, IITJEEClasses, IITJEETuitions inPatna. GetPhoneNumbers, Address, Reviews, Photos, Maps for top Tutorials For IITJEEnear me inPatnaon Justdial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>AGM-1038</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Bansal Classes Patna</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Patna</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Bihar</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>9135699903</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/919135699903</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>info@bansalpatna.com</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bansalpatna.com/</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Tier A (High Value)</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>BestIIT-JEE&amp;NEETCoachinginPatnaAchieve YourBestwith Dedicated Personal GuidancePatna'smost trustedcoachinginstituteforJEE&amp;NEET— since 1981. Bansal ClassesPatnais part of the Bansal network, which has produced 25,000+ IITians &amp; 1,00,000+ Engineers across 73+ centres. FREE BOOST scholarship test for session 2027-28 →</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>AGM-1039</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Top IIT JEE Coaching in Patna With Fees</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Patna</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Bihar</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>8571428571</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/918571428571</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr"/>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>https://bestinpatna.com/top-5-iit-jee-coaching-in-patna/</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Tier A (High Value)</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P39" s="3" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q39" s="3" t="inlineStr">
+        <is>
+          <t>Physics Wallah VidyapeethCoachingCenter,PatnaKankarbagh is a premierinstitutefor students searching forbestIITJEEcoachinginPatnaand also offers preparation forNEETand foundation courses. Strategically located on 4th Floor, Rajeshwar Complex, Kankarbagh Main Rd, Rajendra Nagar,Patna, the center serves students from Rajendra Nagar and nearby areas, making it ideal for those ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>AGM-1040</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Contact GOAL Institute Patna</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Coaching Institute</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Patna</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Bihar</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>6123508700</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/916123508700</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>email@example.com</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goalinstitute.org/contact-us</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Tier A (High Value)</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>Web Search Discovery</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P40" s="3" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>ContactGOALInstitute, the topcoachingcenter inPatnaforNEETand IIT-JEE, and medical preparation. Reach out for admissions, queries, and more.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>AGM-1041</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Unacademy UPSC (YouTube)</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>YouTube / Online Educator</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Online / Pan-India</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr"/>
+      <c r="H41" s="8" t="inlineStr"/>
+      <c r="I41" s="8" t="inlineStr"/>
+      <c r="J41" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/c/UnacademyUPSC</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="L41" s="7" t="inlineStr">
+        <is>
+          <t>Tier C (Nurture)</t>
+        </is>
+      </c>
+      <c r="M41" s="8" t="inlineStr">
+        <is>
+          <t>YouTube Educator Discovery</t>
+        </is>
+      </c>
+      <c r="N41" s="7" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O41" s="7" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P41" s="8" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q41" s="8" t="inlineStr">
+        <is>
+          <t>Welcome to UncademyUPSC, your one-stop solution forUPSCCSEpreparation.India'stop educators will be teaching you daily on this channel. We will cover the entire syllabus, strategy, updates ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>AGM-1042</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>CrashCourse (YouTube)</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>YouTube / Online Educator</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>Online / Pan-India</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr"/>
+      <c r="H42" s="10" t="inlineStr"/>
+      <c r="I42" s="10" t="inlineStr"/>
+      <c r="J42" s="10" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/c/crashcourse</t>
+        </is>
+      </c>
+      <c r="K42" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="L42" s="9" t="inlineStr">
+        <is>
+          <t>Tier C (Nurture)</t>
+        </is>
+      </c>
+      <c r="M42" s="10" t="inlineStr">
+        <is>
+          <t>YouTube Educator Discovery</t>
+        </is>
+      </c>
+      <c r="N42" s="9" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O42" s="9" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P42" s="10" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q42" s="10" t="inlineStr">
+        <is>
+          <t>At Crash Course, we believe that high-quality educational videos should be available to everyone for free! Subscribe for weekly videos from our current courses! The Crash Course team has produced ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>AGM-1043</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Drishti IAS (YouTube)</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>YouTube / Online Educator</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Online / Pan-India</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr"/>
+      <c r="H43" s="8" t="inlineStr"/>
+      <c r="I43" s="8" t="inlineStr"/>
+      <c r="J43" s="8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/c/DrishtiIASvideos/videos</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="L43" s="7" t="inlineStr">
+        <is>
+          <t>Tier C (Nurture)</t>
+        </is>
+      </c>
+      <c r="M43" s="8" t="inlineStr">
+        <is>
+          <t>YouTube Educator Discovery</t>
+        </is>
+      </c>
+      <c r="N43" s="7" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O43" s="7" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P43" s="8" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q43" s="8" t="inlineStr">
+        <is>
+          <t>'Drishti The Vision Foundation,' also known as 'Drishti IAS,' was founded on November 1, 1999. Currently, Drishti IAS has a physical presence across eight cities. It has centres in Delhi (Karol ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>AGM-1044</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>Gohar Khan (YouTube)</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>YouTube / Online Educator</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>Online / Pan-India</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="inlineStr"/>
+      <c r="H44" s="10" t="inlineStr"/>
+      <c r="I44" s="10" t="inlineStr"/>
+      <c r="J44" s="10" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/c/GoharsGuide</t>
+        </is>
+      </c>
+      <c r="K44" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="L44" s="9" t="inlineStr">
+        <is>
+          <t>Tier C (Nurture)</t>
+        </is>
+      </c>
+      <c r="M44" s="10" t="inlineStr">
+        <is>
+          <t>YouTube Educator Discovery</t>
+        </is>
+      </c>
+      <c r="N44" s="9" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="O44" s="9" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="P44" s="10" t="inlineStr">
+        <is>
+          <t>Branded App &amp; Student Ads</t>
+        </is>
+      </c>
+      <c r="Q44" s="10" t="inlineStr">
+        <is>
+          <t>An MIT grad helping you survive college and life! Hi! My name is Gohar Khan, and I graduated from MIT with a BSc in Computer Science, Economics, and Data Science, as well as in Business Analytics ...</t>
         </is>
       </c>
     </row>
@@ -2641,7 +4150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -2750,6 +4259,81 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>Added 12 verified leads to AGMIDI pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-29 02:39:42</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Success (Auto-Run)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Pan-India Coaching Hubs &amp; Creators</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Added 0 verified leads to AGMIDI pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-29 02:39:48</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Success (Auto-Run)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Pan-India Coaching Hubs &amp; Creators</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Added 0 verified leads to AGMIDI pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:58:30</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>19</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Success (Auto-Run)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Pan-India Coaching Hubs &amp; Creators</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Added 19 verified leads to AGMIDI pipeline</t>
         </is>
       </c>
     </row>

</xml_diff>